<commit_message>
Please provide the file changes to generate a commit message.
</commit_message>
<xml_diff>
--- a/OI/A0 Pareto - Ishikawa/Template_Pareto_Chaudronnier.xlsx
+++ b/OI/A0 Pareto - Ishikawa/Template_Pareto_Chaudronnier.xlsx
@@ -8,23 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cfaicentre-my.sharepoint.com/personal/s_jaubert_poleformation-uimmcvdl_fr/Documents/00FC/OI/A0 Pareto - Ishikawa/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="11_E62DBA95E96421727B015E18D07CDFF7B80D98E7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D7FD6843-344E-48CD-BFCD-97A1BCF96E7D}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="11_E62DBA95E96421727B015E18D07CDFF7B80D98E7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{520E0471-0C46-4626-8736-1B79245B46F2}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Modele Vierge" sheetId="1" r:id="rId1"/>
     <sheet name="Activite 2 - Tuyauterie" sheetId="2" r:id="rId2"/>
     <sheet name="Activite 3 - Deux ateliers" sheetId="3" r:id="rId3"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlchart.v1.0" hidden="1">'Activite 3 - Deux ateliers'!$A$5:$A$11</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">'Activite 3 - Deux ateliers'!$B$5:$B$11</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">'Activite 3 - Deux ateliers'!$A$5:$A$11</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">'Activite 3 - Deux ateliers'!$B$5:$B$11</definedName>
-  </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -321,11 +314,11 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -643,12 +636,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -787,11 +780,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
@@ -934,16 +927,18 @@
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="11" max="11" width="28.7109375" customWidth="1"/>
+    <col min="12" max="12" width="20.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
     </row>
     <row r="3" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">

</xml_diff>

<commit_message>
feat: Add Lean "Atelier Cocotte" workshop materials and a Pareto-Ishikawa template.
</commit_message>
<xml_diff>
--- a/OI/A0 Pareto - Ishikawa/Template_Pareto_Chaudronnier.xlsx
+++ b/OI/A0 Pareto - Ishikawa/Template_Pareto_Chaudronnier.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cfaicentre-my.sharepoint.com/personal/s_jaubert_poleformation-uimmcvdl_fr/Documents/00FC/OI/A0 Pareto - Ishikawa/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="11_E62DBA95E96421727B015E18D07CDFF7B80D98E7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{520E0471-0C46-4626-8736-1B79245B46F2}"/>
+  <xr:revisionPtr revIDLastSave="50" documentId="11_E62DBA95E96421727B015E18D07CDFF7B80D98E7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{605B835E-AB6D-4020-A746-167E53F7C4B8}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Modele Vierge" sheetId="1" r:id="rId1"/>
-    <sheet name="Activite 2 - Tuyauterie" sheetId="2" r:id="rId2"/>
-    <sheet name="Activite 3 - Deux ateliers" sheetId="3" r:id="rId3"/>
+    <sheet name="Feuil1" sheetId="4" r:id="rId2"/>
+    <sheet name="Activite 2 - Tuyauterie" sheetId="2" r:id="rId3"/>
+    <sheet name="Activite 3 - Deux ateliers" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="59">
   <si>
     <t>DIAGRAMME DE PARETO - MODELE VIERGE</t>
   </si>
@@ -182,13 +183,43 @@
   </si>
   <si>
     <t>Erreur de reperage</t>
+  </si>
+  <si>
+    <t>type de defaut</t>
+  </si>
+  <si>
+    <t>quantité</t>
+  </si>
+  <si>
+    <t>Porosité (soudure)</t>
+  </si>
+  <si>
+    <t>Caniveau (soudure)</t>
+  </si>
+  <si>
+    <t>Déformation (pliage/soudure)</t>
+  </si>
+  <si>
+    <t>Cote Hors Tolérance (découpe)</t>
+  </si>
+  <si>
+    <t>Rayure (manutention)</t>
+  </si>
+  <si>
+    <t>Fissure (soudure)</t>
+  </si>
+  <si>
+    <t>Fréquence</t>
+  </si>
+  <si>
+    <t>Fréquence Cumulée</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -237,8 +268,36 @@
       <color rgb="FF8E44AD"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF999999"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -261,6 +320,24 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF8E44AD"/>
         <bgColor rgb="FF8E44AD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF3CD"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFEF9F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -288,10 +365,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -314,14 +392,32 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Pourcentage" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -334,6 +430,878 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="fr-FR"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="fr-FR"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Feuil1!$A$2:$A$7</c:f>
+              <c:strCache>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>Porosité (soudure)</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Caniveau (soudure)</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Déformation (pliage/soudure)</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Cote Hors Tolérance (découpe)</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Rayure (manutention)</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Fissure (soudure)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Feuil1!$B$2:$B$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>42</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-B985-42D7-AE4C-94F936ECED71}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="65286416"/>
+        <c:axId val="65287376"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="65286416"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="fr-FR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="65287376"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="65287376"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="fr-FR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="65286416"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="fr-FR"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>997164</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>129945</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>643801</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>64997</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Graphique 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{170C86E4-75FF-CD83-67CC-CDE1F7531164}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
@@ -629,51 +1597,51 @@
     <tabColor rgb="FFE67E22"/>
   </sheetPr>
   <dimension ref="A1:D21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
     <col min="2" max="4" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="13" t="s">
+    <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A10" s="2" t="s">
         <v>7</v>
       </c>
@@ -687,67 +1655,67 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A11" s="3"/>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A12" s="3"/>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A13" s="3"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A14" s="3"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A15" s="3"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A16" s="3"/>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
       <c r="D16" s="4"/>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A17" s="3"/>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
       <c r="D17" s="4"/>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A18" s="3"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A19" s="3"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A20" s="3"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A21" s="5" t="s">
         <v>11</v>
       </c>
@@ -767,36 +1735,167 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC1EFDFC-80EF-46B3-B4F8-F8369B7E5EB6}">
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="26.265625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A1" s="19" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1" s="19" t="s">
+        <v>50</v>
+      </c>
+      <c r="C1" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="D1" s="20" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A2" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="B2" s="16">
+        <v>42</v>
+      </c>
+      <c r="C2" s="18">
+        <f>B2/$B$8</f>
+        <v>0.56756756756756754</v>
+      </c>
+      <c r="D2" s="21">
+        <f>C2</f>
+        <v>0.56756756756756754</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A3" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B3" s="16">
+        <v>13</v>
+      </c>
+      <c r="C3" s="18">
+        <f t="shared" ref="C3:C7" si="0">B3/$B$8</f>
+        <v>0.17567567567567569</v>
+      </c>
+      <c r="D3" s="21">
+        <f>D2+C3</f>
+        <v>0.7432432432432432</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="23.65" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A4" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="B4" s="16">
+        <v>8</v>
+      </c>
+      <c r="C4" s="18">
+        <f t="shared" si="0"/>
+        <v>0.10810810810810811</v>
+      </c>
+      <c r="D4" s="21">
+        <f t="shared" ref="D4:D7" si="1">D3+C4</f>
+        <v>0.85135135135135132</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="27" x14ac:dyDescent="0.45">
+      <c r="A5" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5" s="16">
+        <v>5</v>
+      </c>
+      <c r="C5" s="18">
+        <f t="shared" si="0"/>
+        <v>6.7567567567567571E-2</v>
+      </c>
+      <c r="D5" s="21">
+        <f t="shared" si="1"/>
+        <v>0.91891891891891886</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A6" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="B6" s="16">
+        <v>3</v>
+      </c>
+      <c r="C6" s="18">
+        <f t="shared" si="0"/>
+        <v>4.0540540540540543E-2</v>
+      </c>
+      <c r="D6" s="21">
+        <f t="shared" si="1"/>
+        <v>0.95945945945945943</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A7" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="B7" s="16">
+        <v>3</v>
+      </c>
+      <c r="C7" s="18">
+        <f t="shared" si="0"/>
+        <v>4.0540540540540543E-2</v>
+      </c>
+      <c r="D7" s="21">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="B8">
+        <f>SUM(B2:B7)</f>
+        <v>74</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <tabColor rgb="FFD35400"/>
   </sheetPr>
   <dimension ref="A1:C17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
     <col min="2" max="2" width="40" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="13" t="s">
+    <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" s="7" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" s="7" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" s="8" t="s">
         <v>7</v>
       </c>
@@ -807,7 +1906,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" s="3" t="s">
         <v>16</v>
       </c>
@@ -818,7 +1917,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A8" s="3" t="s">
         <v>18</v>
       </c>
@@ -829,7 +1928,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" s="3" t="s">
         <v>20</v>
       </c>
@@ -840,7 +1939,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A10" s="3" t="s">
         <v>22</v>
       </c>
@@ -851,7 +1950,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A11" s="3" t="s">
         <v>24</v>
       </c>
@@ -862,7 +1961,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A12" s="3" t="s">
         <v>26</v>
       </c>
@@ -873,7 +1972,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A13" s="3" t="s">
         <v>28</v>
       </c>
@@ -884,7 +1983,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A14" s="3" t="s">
         <v>30</v>
       </c>
@@ -895,7 +1994,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A15" s="5" t="s">
         <v>11</v>
       </c>
@@ -904,7 +2003,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A17" s="1" t="s">
         <v>32</v>
       </c>
@@ -917,35 +2016,35 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <tabColor rgb="FF8E44AD"/>
   </sheetPr>
   <dimension ref="A1:E22"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="11" max="11" width="28.7109375" customWidth="1"/>
-    <col min="12" max="12" width="20.7109375" customWidth="1"/>
+    <col min="11" max="11" width="28.73046875" customWidth="1"/>
+    <col min="12" max="12" width="20.73046875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="12" t="s">
+    <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-    </row>
-    <row r="3" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+    </row>
+    <row r="3" spans="1:5" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A3" s="9" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
@@ -953,7 +2052,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A5" s="3" t="s">
         <v>35</v>
       </c>
@@ -961,7 +2060,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A6" s="3" t="s">
         <v>36</v>
       </c>
@@ -969,7 +2068,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A7" s="3" t="s">
         <v>37</v>
       </c>
@@ -977,7 +2076,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A8" s="3" t="s">
         <v>38</v>
       </c>
@@ -985,7 +2084,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A9" s="3" t="s">
         <v>39</v>
       </c>
@@ -993,7 +2092,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A10" s="3" t="s">
         <v>40</v>
       </c>
@@ -1001,7 +2100,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A11" s="3" t="s">
         <v>41</v>
       </c>
@@ -1009,12 +2108,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A14" s="10" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A15" s="11" t="s">
         <v>7</v>
       </c>
@@ -1022,7 +2121,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A16" s="3" t="s">
         <v>43</v>
       </c>
@@ -1030,7 +2129,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A17" s="3" t="s">
         <v>44</v>
       </c>
@@ -1038,7 +2137,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A18" s="3" t="s">
         <v>45</v>
       </c>
@@ -1046,7 +2145,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A19" s="3" t="s">
         <v>46</v>
       </c>
@@ -1054,7 +2153,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A20" s="3" t="s">
         <v>18</v>
       </c>
@@ -1062,7 +2161,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A21" s="3" t="s">
         <v>47</v>
       </c>
@@ -1070,7 +2169,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A22" s="3" t="s">
         <v>48</v>
       </c>

</xml_diff>